<commit_message>
Eksamen: legg til skoleeksamen V26 og rett H25-merking i 9.1-tabellen
Nye filer skole-26-v.pdf, skole-26-v-fasit.pdf og skole-26-v-ekstra.zip
(sistnevnte med sykler.RData). skoleeksamen.xlsx: ny rad for 2026 - Vaar,
og H25-raden rettet fra feilaktig '2026 - høst' til '2025 - høst'.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tidligere-eksamensoppgaver/skoleeksamen.xlsx
+++ b/tidligere-eksamensoppgaver/skoleeksamen.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30131"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\git\met4\tidligere-eksamensoppgaver\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{507CF955-80CE-4A5B-AEFB-27E28A6DD211}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{45DF6B5C-43E6-4771-A636-FC539C0476F2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="390" windowWidth="29010" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="68">
   <si>
     <t>Semester</t>
   </si>
@@ -207,9 +207,6 @@
     <t>[Materiale](tidligere-eksamensoppgaver/skole-25-v-ekstra.zip)</t>
   </si>
   <si>
-    <t>2026 - høst</t>
-  </si>
-  <si>
     <t>[Oppgaveformulering](tidligere-eksamensoppgaver/skole-25-h.pdf)</t>
   </si>
   <si>
@@ -217,14 +214,37 @@
   </si>
   <si>
     <t>[Materiale](tidligere-eksamensoppgaver/skole-25-h-ekstra.zip)</t>
+  </si>
+  <si>
+    <t>2025 - høst</t>
+  </si>
+  <si>
+    <t>2026 - Vår</t>
+  </si>
+  <si>
+    <t>[Oppgaveformulering](tidligere-eksamensoppgaver/skole-26-v.pdf)</t>
+  </si>
+  <si>
+    <t>[Løsningsforslag](tidligere-eksamensoppgaver/skole-26-v-fasit.pdf)</t>
+  </si>
+  <si>
+    <t>[Materiale](tidligere-eksamensoppgaver/skole-26-v-ekstra.zip)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -252,8 +272,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -534,18 +555,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E19"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.06640625" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <dimension ref="A1:E22"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="19" customWidth="1"/>
-    <col min="2" max="2" width="52.46484375" customWidth="1"/>
-    <col min="3" max="3" width="66.06640625" customWidth="1"/>
-    <col min="4" max="4" width="57.53125" customWidth="1"/>
-    <col min="5" max="5" width="56.265625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="8.73046875" customWidth="1"/>
+    <col min="2" max="2" width="52.42578125" customWidth="1"/>
+    <col min="3" max="3" width="66" customWidth="1"/>
+    <col min="4" max="4" width="57.5703125" customWidth="1"/>
+    <col min="5" max="5" width="56.28515625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="8.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -562,7 +583,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -576,7 +597,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>7</v>
       </c>
@@ -590,7 +611,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>10</v>
       </c>
@@ -601,7 +622,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>13</v>
       </c>
@@ -615,7 +636,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>17</v>
       </c>
@@ -629,7 +650,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>20</v>
       </c>
@@ -640,7 +661,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>23</v>
       </c>
@@ -651,7 +672,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>26</v>
       </c>
@@ -662,7 +683,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>29</v>
       </c>
@@ -673,7 +694,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>32</v>
       </c>
@@ -684,7 +705,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>36</v>
       </c>
@@ -695,7 +716,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>39</v>
       </c>
@@ -706,7 +727,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>44</v>
       </c>
@@ -717,7 +738,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>45</v>
       </c>
@@ -728,7 +749,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>48</v>
       </c>
@@ -739,7 +760,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>51</v>
       </c>
@@ -750,7 +771,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>54</v>
       </c>
@@ -764,19 +785,36 @@
         <v>59</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
+        <v>63</v>
+      </c>
+      <c r="B19" t="s">
         <v>60</v>
       </c>
-      <c r="B19" t="s">
+      <c r="C19" t="s">
         <v>61</v>
       </c>
-      <c r="C19" t="s">
+      <c r="E19" t="s">
         <v>62</v>
       </c>
-      <c r="E19" t="s">
-        <v>63</v>
-      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>64</v>
+      </c>
+      <c r="B20" t="s">
+        <v>65</v>
+      </c>
+      <c r="C20" t="s">
+        <v>66</v>
+      </c>
+      <c r="E20" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="C22" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>